<commit_message>
demos: make codescan, compress_tc, gcomp, and tvtools demos run on a clean machine
- compress_tc: install from the checkout instead of running only the main
  ado, so helpers no longer resolve from a stale installed copy
- tvtools: install tvtools and pin white_tableau instead of relying on a
  preinstalled copy and the caller's scheme; README recipe says so
- gcomp: per-run temp PLUS directory so concurrent demos no longer collide;
  refreshes the stale component_models.md
- codescan: resolve tc_schemes before sandboxing and use white_tableau;
  stop clipping the largest bar label
</commit_message>
<xml_diff>
--- a/gcomp/demo/demo_gcomptab.xlsx
+++ b/gcomp/demo/demo_gcomptab.xlsx
@@ -125,7 +125,7 @@
     <t>0.700***</t>
   </si>
   <si>
-    <t>[0.497, 0.903]</t>
+    <t>[0.496, 0.904]</t>
   </si>
   <si>
     <t>&lt;0.001</t>
@@ -167,16 +167,16 @@
     <t>[-0.204, 0.056]</t>
   </si>
   <si>
-    <t>0.263</t>
+    <t>0.264</t>
   </si>
   <si>
     <t>0.089</t>
   </si>
   <si>
-    <t>[-0.052, 0.229]</t>
+    <t>[-0.052, 0.230]</t>
   </si>
   <si>
-    <t>0.216</t>
+    <t>0.217</t>
   </si>
   <si>
     <t>m</t>
@@ -185,7 +185,7 @@
     <t>0.755***</t>
   </si>
   <si>
-    <t>[0.648, 0.861]</t>
+    <t>[0.648, 0.862]</t>
   </si>
   <si>
     <t>N</t>

</xml_diff>